<commit_message>
Atualiza categorias dos produtos
</commit_message>
<xml_diff>
--- a/dados/Dados.xlsx
+++ b/dados/Dados.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fastshop Arica\OneDrive\Documents\MeuSiteAmigurumi\dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fastshop Arica\OneDrive\Documents\ateliebarbaradias\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="190">
   <si>
     <t>ID</t>
   </si>
@@ -126,9 +126,6 @@
     <t>Embalagem</t>
   </si>
   <si>
-    <t>profundidade (cm)</t>
-  </si>
-  <si>
     <t>Boneca Buque Flor</t>
   </si>
   <si>
@@ -198,9 +195,6 @@
     <t>Kit Bebe Ursinho com Naninha</t>
   </si>
   <si>
-    <t>Brinquedi</t>
-  </si>
-  <si>
     <t>kit-bebe-ursinho-com-naninha</t>
   </si>
   <si>
@@ -318,9 +312,6 @@
     <t>Tapete Hexagonal Verde</t>
   </si>
   <si>
-    <t>Decorção</t>
-  </si>
-  <si>
     <t>tapete-hexagonal-verde</t>
   </si>
   <si>
@@ -595,6 +586,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Confeccionado com fio 100% e enchimento hipoalergênico. Altura 28cm.</t>
+  </si>
+  <si>
+    <t>Profundidade (cm)</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +995,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
@@ -1022,7 +1016,7 @@
         <v>11</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>35</v>
+        <v>189</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>34</v>
@@ -1039,13 +1033,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>108</v>
       </c>
       <c r="E2" s="4">
         <v>150</v>
@@ -1081,7 +1075,7 @@
         <v>5</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -1089,13 +1083,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E3" s="4">
         <v>299</v>
@@ -1131,7 +1125,7 @@
         <v>2</v>
       </c>
       <c r="Q3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
@@ -1139,13 +1133,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E4" s="4">
         <v>219</v>
@@ -1181,7 +1175,7 @@
         <v>4</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
@@ -1189,13 +1183,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E5" s="4">
         <v>260</v>
@@ -1231,7 +1225,7 @@
         <v>5</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
@@ -1239,13 +1233,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E6" s="4">
         <v>200</v>
@@ -1281,7 +1275,7 @@
         <v>3</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
@@ -1289,13 +1283,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E7" s="4">
         <v>260</v>
@@ -1331,7 +1325,7 @@
         <v>4</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
@@ -1339,13 +1333,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E8" s="4">
         <v>210</v>
@@ -1381,7 +1375,7 @@
         <v>4</v>
       </c>
       <c r="Q8" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -1431,7 +1425,7 @@
         <v>2</v>
       </c>
       <c r="Q9" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
@@ -1439,13 +1433,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E10" s="4">
         <v>130</v>
@@ -1481,7 +1475,7 @@
         <v>4</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
@@ -1492,10 +1486,10 @@
         <v>20</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="E11" s="4">
         <v>100</v>
@@ -1531,7 +1525,7 @@
         <v>2</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
@@ -1539,13 +1533,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E12" s="4">
         <v>90</v>
@@ -1581,7 +1575,7 @@
         <v>5</v>
       </c>
       <c r="Q12" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
@@ -1592,7 +1586,7 @@
         <v>21</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>22</v>
@@ -1631,7 +1625,7 @@
         <v>5</v>
       </c>
       <c r="Q13" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
@@ -1639,13 +1633,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E14" s="4">
         <v>8</v>
@@ -1681,7 +1675,7 @@
         <v>3</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -1689,13 +1683,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E15" s="4">
         <v>8</v>
@@ -1731,7 +1725,7 @@
         <v>5</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -1739,13 +1733,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E16" s="4">
         <v>8</v>
@@ -1781,7 +1775,7 @@
         <v>7</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
@@ -1789,13 +1783,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E17" s="4">
         <v>10</v>
@@ -1831,7 +1825,7 @@
         <v>3</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
@@ -1839,13 +1833,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E18" s="4">
         <v>75</v>
@@ -1881,7 +1875,7 @@
         <v>3</v>
       </c>
       <c r="Q18" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
@@ -1892,10 +1886,10 @@
         <v>24</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E19" s="4">
         <v>80</v>
@@ -1931,7 +1925,7 @@
         <v>2</v>
       </c>
       <c r="Q19" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
@@ -1942,7 +1936,7 @@
         <v>25</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>27</v>
@@ -1981,7 +1975,7 @@
         <v>4</v>
       </c>
       <c r="Q20" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
@@ -2031,7 +2025,7 @@
         <v>5</v>
       </c>
       <c r="Q21" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
@@ -2039,13 +2033,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E22" s="4">
         <v>300</v>
@@ -2081,7 +2075,7 @@
         <v>4</v>
       </c>
       <c r="Q22" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
@@ -2089,13 +2083,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E23" s="4">
         <v>300</v>
@@ -2131,7 +2125,7 @@
         <v>4</v>
       </c>
       <c r="Q23" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
@@ -2139,13 +2133,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E24" s="4">
         <v>70</v>
@@ -2181,7 +2175,7 @@
         <v>1</v>
       </c>
       <c r="Q24" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
@@ -2189,13 +2183,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E25" s="4">
         <v>100</v>
@@ -2231,7 +2225,7 @@
         <v>2</v>
       </c>
       <c r="Q25" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
@@ -2239,13 +2233,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>60</v>
       </c>
       <c r="E26" s="4">
         <v>250</v>
@@ -2281,7 +2275,7 @@
         <v>3</v>
       </c>
       <c r="Q26" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
@@ -2289,13 +2283,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E27" s="4">
         <v>190</v>
@@ -2331,7 +2325,7 @@
         <v>2</v>
       </c>
       <c r="Q27" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.3">
@@ -2339,13 +2333,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>90</v>
       </c>
       <c r="E28" s="4">
         <v>210</v>
@@ -2381,7 +2375,7 @@
         <v>3</v>
       </c>
       <c r="Q28" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.3">
@@ -2389,13 +2383,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E29" s="4">
         <v>100</v>
@@ -2431,7 +2425,7 @@
         <v>3</v>
       </c>
       <c r="Q29" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.3">
@@ -2439,13 +2433,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E30" s="4">
         <v>200</v>
@@ -2481,7 +2475,7 @@
         <v>3</v>
       </c>
       <c r="Q30" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.3">
@@ -2489,13 +2483,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E31" s="4">
         <v>190</v>
@@ -2531,7 +2525,7 @@
         <v>4</v>
       </c>
       <c r="Q31" s="2" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.3">
@@ -2539,13 +2533,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E32" s="4">
         <v>180</v>
@@ -2581,7 +2575,7 @@
         <v>6</v>
       </c>
       <c r="Q32" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.3">
@@ -2589,13 +2583,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E33" s="4">
         <v>200</v>
@@ -2616,7 +2610,7 @@
         <v>16</v>
       </c>
       <c r="K33" s="1">
-        <v>1100</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="L33" s="1">
         <v>35</v>
@@ -2631,7 +2625,7 @@
         <v>3</v>
       </c>
       <c r="Q33" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.3">
@@ -2639,13 +2633,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E34" s="4">
         <v>45</v>
@@ -2681,7 +2675,7 @@
         <v>2</v>
       </c>
       <c r="Q34" s="2" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.3">
@@ -2689,13 +2683,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E35" s="4">
         <v>30</v>
@@ -2731,7 +2725,7 @@
         <v>2</v>
       </c>
       <c r="Q35" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.3">
@@ -2739,13 +2733,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E36" s="4">
         <v>30</v>
@@ -2781,7 +2775,7 @@
         <v>2</v>
       </c>
       <c r="Q36" s="2" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.3">
@@ -2789,13 +2783,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E37" s="4">
         <v>50</v>
@@ -2831,7 +2825,7 @@
         <v>3</v>
       </c>
       <c r="Q37" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.3">
@@ -2839,13 +2833,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="E38" s="4">
         <v>310</v>
@@ -2881,7 +2875,7 @@
         <v>4</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.3">
@@ -2889,13 +2883,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E39" s="4">
         <v>190</v>
@@ -2931,7 +2925,7 @@
         <v>6</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
@@ -2945,7 +2939,7 @@
         <v>31</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E40" s="4">
         <v>210</v>
@@ -2981,7 +2975,7 @@
         <v>5</v>
       </c>
       <c r="Q40" s="2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.3">
@@ -2989,13 +2983,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E41" s="4">
         <v>50</v>
@@ -3031,7 +3025,7 @@
         <v>2</v>
       </c>
       <c r="Q41" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.3">
@@ -3039,13 +3033,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E42" s="4">
         <v>50</v>
@@ -3081,7 +3075,7 @@
         <v>3</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="43" spans="1:17" x14ac:dyDescent="0.3">
@@ -3089,13 +3083,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E43" s="4">
         <v>50</v>
@@ -3131,7 +3125,7 @@
         <v>3</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.3">
@@ -3139,13 +3133,13 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E44" s="4">
         <v>180</v>
@@ -3181,7 +3175,7 @@
         <v>2</v>
       </c>
       <c r="Q44" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="45" spans="1:17" x14ac:dyDescent="0.3">
@@ -3189,13 +3183,13 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E45" s="4">
         <v>190</v>
@@ -3231,7 +3225,7 @@
         <v>4</v>
       </c>
       <c r="Q45" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.3">
@@ -3239,13 +3233,13 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E46" s="4">
         <v>250</v>
@@ -3281,7 +3275,7 @@
         <v>3</v>
       </c>
       <c r="Q46" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.3">
@@ -3289,13 +3283,13 @@
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E47" s="4">
         <v>200</v>
@@ -3331,7 +3325,7 @@
         <v>5</v>
       </c>
       <c r="Q47" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.3">
@@ -3339,13 +3333,13 @@
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E48" s="4">
         <v>100</v>
@@ -3381,7 +3375,7 @@
         <v>3</v>
       </c>
       <c r="Q48" s="1" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.3">
@@ -3389,13 +3383,13 @@
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>99</v>
+        <v>26</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E49" s="4">
         <v>100</v>
@@ -3431,7 +3425,7 @@
         <v>3</v>
       </c>
       <c r="Q49" s="1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.3">
@@ -3439,13 +3433,13 @@
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E50" s="4">
         <v>95</v>
@@ -3481,7 +3475,7 @@
         <v>5</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.3">
@@ -3489,13 +3483,13 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E51" s="4">
         <v>195</v>
@@ -3531,7 +3525,7 @@
         <v>3</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="52" spans="1:17" x14ac:dyDescent="0.3">
@@ -3539,13 +3533,13 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E52" s="4">
         <v>80</v>
@@ -3581,7 +3575,7 @@
         <v>4</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="53" spans="1:17" x14ac:dyDescent="0.3">
@@ -3589,13 +3583,13 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E53" s="4">
         <v>80</v>
@@ -3631,7 +3625,7 @@
         <v>5</v>
       </c>
       <c r="Q53" s="1" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="54" spans="1:17" x14ac:dyDescent="0.3">
@@ -3639,13 +3633,13 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E54" s="4">
         <v>140</v>
@@ -3681,7 +3675,7 @@
         <v>4</v>
       </c>
       <c r="Q54" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="55" spans="1:17" x14ac:dyDescent="0.3">
@@ -3689,10 +3683,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D55" s="1" t="s">
         <v>19</v>
@@ -3731,7 +3725,7 @@
         <v>10</v>
       </c>
       <c r="Q55" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="56" spans="1:17" x14ac:dyDescent="0.3">
@@ -3781,7 +3775,7 @@
         <v>6</v>
       </c>
       <c r="Q56" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="57" spans="1:17" x14ac:dyDescent="0.3">
@@ -3789,13 +3783,13 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E57" s="4">
         <v>60</v>
@@ -3831,7 +3825,7 @@
         <v>3</v>
       </c>
       <c r="Q57" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="58" spans="1:17" x14ac:dyDescent="0.3">
@@ -3839,13 +3833,13 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E58" s="4">
         <v>90</v>
@@ -3869,7 +3863,7 @@
         <v>0.222</v>
       </c>
       <c r="L58" s="1">
-        <v>323</v>
+        <v>32</v>
       </c>
       <c r="M58" s="1">
         <v>10</v>
@@ -3881,7 +3875,7 @@
         <v>4</v>
       </c>
       <c r="Q58" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adicionados novos produtos e fotos
</commit_message>
<xml_diff>
--- a/dados/Dados.xlsx
+++ b/dados/Dados.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="216">
   <si>
     <t>ID</t>
   </si>
@@ -589,6 +589,84 @@
   </si>
   <si>
     <t>Profundidade (cm)</t>
+  </si>
+  <si>
+    <t>Sousplat Azul com Dourado</t>
+  </si>
+  <si>
+    <t>sousplat-azul-dourado</t>
+  </si>
+  <si>
+    <t>Uma peça que une beleza e personalidade á sua mesa. Diâmetro: 40cm</t>
+  </si>
+  <si>
+    <t>Sousplat Marrom</t>
+  </si>
+  <si>
+    <t>sousplat-marrom</t>
+  </si>
+  <si>
+    <t>Uma peça que une beleza e personalidade á sua mesa. Diâmetro: 44cm</t>
+  </si>
+  <si>
+    <t>Sousplat rosa</t>
+  </si>
+  <si>
+    <t>sousplat-rosa</t>
+  </si>
+  <si>
+    <t>Uma peça que une beleza e personalidade á sua mesa. Diâmetro: 34cm</t>
+  </si>
+  <si>
+    <t>Kit Sousplat Encanto</t>
+  </si>
+  <si>
+    <t>Uma peça que une beleza e personalidade á sua mesa. Diâmetro: 40cm, porta copo: 14cm diâm.,  porta guardanapo: 7cm diâm., caminho: 1050 X 37com.</t>
+  </si>
+  <si>
+    <t>Kit Sousplat Flor</t>
+  </si>
+  <si>
+    <t>Uma peça que une beleza e personalidade á sua mesa. Diâmetro: 36cm, porta copo: 16cm</t>
+  </si>
+  <si>
+    <t>Sousplat Azul Marinho</t>
+  </si>
+  <si>
+    <t>sousplat-azul-marinho</t>
+  </si>
+  <si>
+    <t>Uma peça que une beleza e personalidade á sua mesa. Diâmetro: 38cm</t>
+  </si>
+  <si>
+    <t>Sousplat verde</t>
+  </si>
+  <si>
+    <t>sousplat-verde</t>
+  </si>
+  <si>
+    <t>Sousplat Caqui</t>
+  </si>
+  <si>
+    <t>sousplat-bege-caqui</t>
+  </si>
+  <si>
+    <t>Uma peça que une beleza e personalidade á sua mesa. Diâmetro: 36cm</t>
+  </si>
+  <si>
+    <t>Porta Copo ou Xícara</t>
+  </si>
+  <si>
+    <t>porta-copo-xicara-flor</t>
+  </si>
+  <si>
+    <t>Porta copo ou xícara Diâmetro: 16cm</t>
+  </si>
+  <si>
+    <t>kit-sousplat-natural-encanto</t>
+  </si>
+  <si>
+    <t>kit-sousplat-flor-marrom-natural</t>
   </si>
 </sst>
 </file>
@@ -958,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q58"/>
+  <dimension ref="A1:Q67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -970,7 +1048,8 @@
     <col min="12" max="12" width="11.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="8.88671875" style="1"/>
+    <col min="15" max="15" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.88671875" style="1"/>
     <col min="17" max="17" width="255.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="18" max="16384" width="8.88671875" style="1"/>
   </cols>
@@ -3876,6 +3955,456 @@
       </c>
       <c r="Q58" t="s">
         <v>188</v>
+      </c>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A59" s="1">
+        <v>58</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E59" s="4">
+        <v>45</v>
+      </c>
+      <c r="F59" s="1">
+        <v>1</v>
+      </c>
+      <c r="G59" s="1">
+        <v>15</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K59" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="L59" s="1">
+        <v>35</v>
+      </c>
+      <c r="M59" s="1">
+        <v>8</v>
+      </c>
+      <c r="N59" s="1">
+        <v>30</v>
+      </c>
+      <c r="P59" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q59" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A60" s="1">
+        <v>59</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E60" s="4">
+        <v>38</v>
+      </c>
+      <c r="F60" s="1">
+        <v>1</v>
+      </c>
+      <c r="G60" s="1">
+        <v>15</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K60" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="L60" s="1">
+        <v>35</v>
+      </c>
+      <c r="M60" s="1">
+        <v>8</v>
+      </c>
+      <c r="N60" s="1">
+        <v>30</v>
+      </c>
+      <c r="P60" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q60" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
+        <v>60</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="E61" s="4">
+        <v>41</v>
+      </c>
+      <c r="F61" s="1">
+        <v>1</v>
+      </c>
+      <c r="G61" s="1">
+        <v>15</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J61" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K61" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="L61" s="1">
+        <v>35</v>
+      </c>
+      <c r="M61" s="1">
+        <v>8</v>
+      </c>
+      <c r="N61" s="1">
+        <v>30</v>
+      </c>
+      <c r="P61" s="1">
+        <v>3</v>
+      </c>
+      <c r="Q61" s="1" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>61</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="E62" s="4">
+        <v>180</v>
+      </c>
+      <c r="F62" s="1">
+        <v>1</v>
+      </c>
+      <c r="G62" s="1">
+        <v>25</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I62" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K62" s="1">
+        <v>0.67500000000000004</v>
+      </c>
+      <c r="L62" s="1">
+        <v>35</v>
+      </c>
+      <c r="M62" s="1">
+        <v>8</v>
+      </c>
+      <c r="N62" s="1">
+        <v>30</v>
+      </c>
+      <c r="P62" s="1">
+        <v>6</v>
+      </c>
+      <c r="Q62" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>62</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E63" s="4">
+        <v>70</v>
+      </c>
+      <c r="F63" s="1">
+        <v>1</v>
+      </c>
+      <c r="G63" s="1">
+        <v>25</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J63" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K63" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="L63" s="1">
+        <v>35</v>
+      </c>
+      <c r="M63" s="1">
+        <v>8</v>
+      </c>
+      <c r="N63" s="1">
+        <v>30</v>
+      </c>
+      <c r="P63" s="1">
+        <v>5</v>
+      </c>
+      <c r="Q63" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
+        <v>63</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="E64" s="4">
+        <v>35</v>
+      </c>
+      <c r="F64" s="1">
+        <v>1</v>
+      </c>
+      <c r="G64" s="1">
+        <v>15</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I64" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J64" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K64" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="L64" s="1">
+        <v>35</v>
+      </c>
+      <c r="M64" s="1">
+        <v>8</v>
+      </c>
+      <c r="N64" s="1">
+        <v>30</v>
+      </c>
+      <c r="P64" s="1">
+        <v>5</v>
+      </c>
+      <c r="Q64" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>64</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="E65" s="4">
+        <v>30</v>
+      </c>
+      <c r="F65" s="1">
+        <v>1</v>
+      </c>
+      <c r="G65" s="1">
+        <v>15</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I65" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J65" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K65" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="L65" s="1">
+        <v>35</v>
+      </c>
+      <c r="M65" s="1">
+        <v>8</v>
+      </c>
+      <c r="N65" s="1">
+        <v>30</v>
+      </c>
+      <c r="P65" s="1">
+        <v>4</v>
+      </c>
+      <c r="Q65" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
+        <v>65</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E66" s="4">
+        <v>35</v>
+      </c>
+      <c r="F66" s="1">
+        <v>1</v>
+      </c>
+      <c r="G66" s="1">
+        <v>15</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J66" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K66" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="L66" s="1">
+        <v>35</v>
+      </c>
+      <c r="M66" s="1">
+        <v>8</v>
+      </c>
+      <c r="N66" s="1">
+        <v>30</v>
+      </c>
+      <c r="P66" s="1">
+        <v>4</v>
+      </c>
+      <c r="Q66" s="1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
+        <v>66</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="E67" s="4">
+        <v>18</v>
+      </c>
+      <c r="F67" s="1">
+        <v>1</v>
+      </c>
+      <c r="G67" s="1">
+        <v>8</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K67" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="L67" s="1">
+        <v>16</v>
+      </c>
+      <c r="M67" s="1">
+        <v>5</v>
+      </c>
+      <c r="N67" s="1">
+        <v>16</v>
+      </c>
+      <c r="P67" s="1">
+        <v>3</v>
+      </c>
+      <c r="Q67" s="1" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>